<commit_message>
Pre Market Fri 2026-06-26
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-06-26.xlsx
+++ b/market-prep/Pre Market 2026-06-26.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29397,92</t>
+          <t>29418,67</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>51920,61</t>
+          <t>51920,63</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4028,13</t>
+          <t>4028,17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>57,86</t>
+          <t>57,90</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1599,50</t>
+          <t>1600,29</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>75,46</t>
+          <t>75,34</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>59503,99</t>
+          <t>59513,89</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1564,77</t>
+          <t>1565,01</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2,52%</t>
+          <t>2,63%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7352,28</t>
+          <t>7348,28</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>